<commit_message>
Log pipeline_history on any successful run, diversify duplicated model descriptions
- pipeline_history.jsonl no longer requires a scheduled-trigger run;
  email-sent success is now the only condition, so manual/chat-driven
  runs get recorded too.
- hf-refine's description-writing guidance now asks for varied phrasing
  (not always ending in "~에 적합") and requires same-family model
  variants (same base model, different size/quant/format) to carry a
  distinguishing detail instead of an identical copy-pasted sentence.
- Rewrote the 102 existing model descriptions that were exact
  duplicates across 33 model-family groups, using already-known
  fields (parameter size, precision/quant, version) to differentiate
  them without fabricating new claims. Regenerated the excel.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/huggingface_models_2026-07-20.xlsx
+++ b/output/huggingface_models_2026-07-20.xlsx
@@ -616,7 +616,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>GRPO로 다중홉 공간추론에 특화 학습되어 순차적 위치·방향 추론 질의응답에 적합</t>
+          <t>GRPO로 다중홉 공간추론에 특화 학습한 32B 모델, 순차적 위치·방향 추론 질의응답에 적합</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -705,7 +705,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>GRPO로 다중홉 공간추론에 특화 학습되어 순차적 위치·방향 추론 질의응답에 적합</t>
+          <t>GRPO로 다중홉 공간추론에 특화 학습한 4B 모델, 순차적 위치·방향 추론 질의응답에 적합</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -794,7 +794,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>GRPO로 다중홉 공간추론에 특화 학습되어 순차적 위치·방향 추론 질의응답에 적합</t>
+          <t>GRPO로 다중홉 공간추론에 특화 학습한 8B 모델, 순차적 위치·방향 추론 질의응답에 적합</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Gemma 기반 VLM에 이미지 안전분류(20종) 기능을 내장, 유해 콘텐츠 탐지·모더레이션에 적합</t>
+          <t>Gemma 12B 기반 VLM에 이미지 안전분류(20종) 기능을 내장, 유해 콘텐츠 탐지·모더레이션에 적합</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -972,7 +972,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Gemma 기반 VLM에 이미지 안전분류(20종) 기능을 내장, 유해 콘텐츠 탐지·모더레이션에 적합</t>
+          <t>Gemma 27B 기반 VLM에 이미지 안전분류(20종) 기능을 내장, 유해 콘텐츠 탐지·모더레이션에 적합</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1061,7 +1061,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Qwen2.5-VL 기반에 이미지 안전분류(20종) 기능을 내장, 유해 콘텐츠 탐지·모더레이션에 적합</t>
+          <t>Qwen2.5-VL 32B 기반에 이미지 안전분류(20종) 기능을 내장, 유해 콘텐츠 탐지·모더레이션에 적합</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Qwen2.5-VL 기반에 이미지 안전분류(20종) 기능을 내장, 유해 콘텐츠 탐지·모더레이션에 적합</t>
+          <t>Qwen2.5-VL 7B 기반에 이미지 안전분류(20종) 기능을 내장, 유해 콘텐츠 탐지·모더레이션에 적합</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1961,7 +1961,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>mT5 인코더와 Code Llama를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
+          <t>mT5 인코더와 Code Llama(약 15B)를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2046,7 +2046,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>mT5 인코더와 Code Llama를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
+          <t>mT5 인코더와 Code Llama(약 20B)를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2131,7 +2131,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>mT5 인코더와 Code Llama를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
+          <t>mT5 인코더와 Code Llama(약 9B)를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>mT5 인코더와 대상 LM을 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
+          <t>mT5 인코더와 Llama2(약 9B)를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>mT5 인코더와 대상 LM을 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
+          <t>mT5 인코더와 Llemma(약 9B)를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>mT5 인코더와 대상 LM을 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
+          <t>mT5 인코더와 MetaMath(약 15B)를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2471,7 +2471,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>mT5 인코더와 대상 LM을 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
+          <t>mT5 인코더와 MetaMath(약 20B)를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2556,7 +2556,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>mT5 인코더와 대상 LM을 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
+          <t>mT5 인코더와 MetaMath(약 9B)를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2641,7 +2641,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>mT5 인코더와 대상 LM을 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
+          <t>mT5 인코더와 Orca2(약 15B)를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2726,7 +2726,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>mT5 인코더와 대상 LM을 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
+          <t>mT5 인코더와 Orca2(약 20B)를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2811,7 +2811,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>mT5 인코더와 대상 LM을 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
+          <t>mT5 인코더와 Orca2(약 9B)를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2896,7 +2896,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>CoT Collection 184만 rationale 학습, Flan-T5보다 CoT 추론 우수해 제로샷 과제 해결에 적합</t>
+          <t>CoT Collection 184만 rationale로 학습한 11B 모델, Flan-T5보다 CoT 추론 우수해 제로샷 과제에 적합</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2981,7 +2981,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>CoT Collection 184만 rationale 학습, Flan-T5보다 CoT 추론 우수해 제로샷 과제 해결에 적합</t>
+          <t>CoT Collection 184만 rationale로 학습한 3B 모델, Flan-T5보다 CoT 추론 우수해 제로샷 과제에 적합</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>문서 이해·한국어 맥락 추론에서 동급 최고 성능인 비전언어모델, 한국어 문서 분석에 적합</t>
+          <t>AWQ 4비트로 양자화한 EXAONE-4.5 VLM, 문서 이해·한국어 맥락 추론에서 동급 최고 성능, 한국어 문서 분석에 적합</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -3367,7 +3367,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>문서 이해·한국어 맥락 추론에서 동급 최고 성능인 비전언어모델, 한국어 문서 분석에 적합</t>
+          <t>FP8로 양자화한 EXAONE-4.5 VLM, 문서 이해·한국어 맥락 추론에서 동급 최고 성능, 한국어 문서 분석에 적합</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3470,7 +3470,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>문서 이해·한국어 맥락 추론에서 동급 최고 성능인 비전언어모델, 한국어 문서 분석에 적합</t>
+          <t>GGUF로 양자화한 EXAONE-4.5 VLM, 문서 이해·한국어 맥락 추론에서 동급 최고 성능, 한국어 문서 분석에 적합</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -4060,7 +4060,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>고성능 32B 모델을 AWQ 4비트로 양자화해 메모리 절약하며 배포 가능</t>
+          <t>EXAONE-3.5 32B 인스트럭트를 AWQ 4비트로 양자화해 메모리 절약하며 배포 가능</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -5315,7 +5315,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>고성능 32B 모델을 AWQ 4비트로 양자화해 메모리 절약하며 배포 가능</t>
+          <t>EXAONE-4.0 32B를 AWQ 4비트로 양자화해 메모리 절약하며 배포 가능</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -7139,7 +7139,7 @@
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
-          <t>문장 전체 없이 실시간 스트리밍으로 대화 음성을 생성해 실시간 음성 대화 시스템에 적합</t>
+          <t>문장 전체 없이 실시간 스트리밍으로 대화 음성을 생성하는 1B 모델, 실시간 음성 대화 시스템에 적합</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -7216,7 +7216,7 @@
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
-          <t>문장 전체 없이 실시간 스트리밍으로 대화 음성을 생성해 실시간 음성 대화 시스템에 적합</t>
+          <t>문장 전체 없이 실시간 스트리밍으로 대화 음성을 생성하는 2B 모델, 실시간 음성 대화 시스템에 적합</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -7297,7 +7297,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>대화체 음성을 실시간에 가깝게 생성하고 웃음·기침 등 비언어적 표현까지 지원, 리서치·교육용 대화형 TTS에 적합</t>
+          <t>대화체 음성을 실시간에 가깝게 생성, 웃음·기침 등 비언어적 표현까지 지원하는 리서치·교육용 대화형 TTS 0626 개정판</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -7382,7 +7382,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>대화체 음성을 실시간에 가깝게 생성하고 웃음·기침 등 비언어적 표현까지 지원, 리서치·교육용 대화형 TTS에 적합</t>
+          <t>대화체 음성을 실시간에 가깝게 생성, 웃음·기침 등 비언어적 표현까지 지원하는 리서치·교육용 대화형 TTS 초기판</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -8692,7 +8692,7 @@
       <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr">
         <is>
-          <t>MLC-LLM·WebLLM에서 바로 구동 가능한 포맷으로 변환해 온디바이스·웹 배포에 적합</t>
+          <t>Vicuna 프루닝 모델을 MLC 포맷(FP16)으로 변환한 1.5B 버전, 온디바이스·웹 배포에 적합</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -8773,7 +8773,7 @@
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
-          <t>MLC-LLM·WebLLM에서 바로 구동 가능한 포맷으로 변환해 온디바이스·웹 배포에 적합</t>
+          <t>Vicuna 프루닝 모델을 MLC용 INT4(q4f16_0)로 양자화한 1.5B 버전, 온디바이스·웹 배포에 적합</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -8854,7 +8854,7 @@
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
-          <t>MLC-LLM·WebLLM에서 바로 구동 가능한 포맷으로 변환해 온디바이스·웹 배포에 적합</t>
+          <t>Vicuna 프루닝 모델을 MLC용 INT4(q4f16_1)로 양자화한 1.5B 버전, 온디바이스·웹 배포에 적합</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -8935,7 +8935,7 @@
       <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
-          <t>MLC-LLM·WebLLM에서 바로 구동 가능한 포맷으로 변환해 온디바이스·웹 배포에 적합</t>
+          <t>Vicuna 프루닝 모델을 MLC 포맷(FP16)으로 변환한 2.7B 버전, 온디바이스·웹 배포에 적합</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -9016,7 +9016,7 @@
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
-          <t>MLC-LLM·WebLLM에서 바로 구동 가능한 포맷으로 변환해 온디바이스·웹 배포에 적합</t>
+          <t>Vicuna 프루닝 모델을 MLC용 INT4(q4f16_0)로 양자화한 2.7B 버전, 온디바이스·웹 배포에 적합</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -9097,7 +9097,7 @@
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
-          <t>MLC-LLM·WebLLM에서 바로 구동 가능한 포맷으로 변환해 온디바이스·웹 배포에 적합</t>
+          <t>Vicuna 프루닝 모델을 MLC용 INT4(q4f16_1)로 양자화한 2.7B 버전, 온디바이스·웹 배포에 적합</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -9178,7 +9178,7 @@
       <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
-          <t>MLC-LLM·WebLLM에서 바로 구동 가능한 포맷으로 변환해 온디바이스·웹 배포에 적합</t>
+          <t>Vicuna 프루닝 모델을 MLC 포맷(FP16)으로 변환한 3.7B 버전, 온디바이스·웹 배포에 적합</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -9259,7 +9259,7 @@
       <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
-          <t>MLC-LLM·WebLLM에서 바로 구동 가능한 포맷으로 변환해 온디바이스·웹 배포에 적합</t>
+          <t>Vicuna 프루닝 모델을 MLC용 INT4(q4f16_0)로 양자화한 3.7B 버전, 온디바이스·웹 배포에 적합</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -9340,7 +9340,7 @@
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
-          <t>MLC-LLM·WebLLM에서 바로 구동 가능한 포맷으로 변환해 온디바이스·웹 배포에 적합</t>
+          <t>Vicuna 프루닝 모델을 MLC용 INT4(q4f16_1)로 양자화한 3.7B 버전, 온디바이스·웹 배포에 적합</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -9421,7 +9421,7 @@
       <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
-          <t>MLC-LLM·WebLLM에서 바로 구동 가능한 포맷으로 변환해 온디바이스·웹 배포에 적합</t>
+          <t>Vicuna 프루닝 모델을 MLC 포맷(FP16)으로 변환한 5.5B 버전, 온디바이스·웹 배포에 적합</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -9502,7 +9502,7 @@
       <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
-          <t>MLC-LLM·WebLLM에서 바로 구동 가능한 포맷으로 변환해 온디바이스·웹 배포에 적합</t>
+          <t>Vicuna 프루닝 모델을 MLC용 INT4(q4f16_0)로 양자화한 5.5B 버전, 온디바이스·웹 배포에 적합</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -9583,7 +9583,7 @@
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr">
         <is>
-          <t>MLC-LLM·WebLLM에서 바로 구동 가능한 포맷으로 변환해 온디바이스·웹 배포에 적합</t>
+          <t>Vicuna 프루닝 모델을 MLC용 INT4(q4f16_1)로 양자화한 5.5B 버전, 온디바이스·웹 배포에 적합</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -9668,7 +9668,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>Vicuna-7B를 프루닝·LoRA로 경량화, GPU 1장으로 수 시간 내 저비용 재학습 가능</t>
+          <t>Vicuna-7B를 프루닝·LoRA로 경량화한 1.5B 버전, GPU 1장으로 수 시간 내 저비용 재학습 가능</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -9757,7 +9757,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>Vicuna-7B를 프루닝·LoRA로 경량화, GPU 1장으로 수 시간 내 저비용 재학습 가능</t>
+          <t>Vicuna-7B를 프루닝·LoRA로 경량화한 2.7B 버전, GPU 1장으로 수 시간 내 저비용 재학습 가능</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -9846,7 +9846,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Vicuna-7B를 프루닝·LoRA로 경량화, GPU 1장으로 수 시간 내 저비용 재학습 가능</t>
+          <t>Vicuna-7B를 프루닝·LoRA로 경량화한 3.7B 버전, GPU 1장으로 수 시간 내 저비용 재학습 가능</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -10024,7 +10024,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>SD-v2.1-base를 지식증류로 압축, 배치 축소로 학습 속도를 높인 경량 텍스트-이미지 모델</t>
+          <t>SD-v2.1-base를 지식증류로 압축한 Base 크기 경량 텍스트-이미지 모델, 배치 축소로 학습 속도 향상</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -10109,7 +10109,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>SD-v2.1-base를 지식증류로 압축, 배치 축소로 학습 속도를 높인 경량 텍스트-이미지 모델</t>
+          <t>SD-v2.1-base를 지식증류로 압축한 Small 크기 경량 텍스트-이미지 모델, 배치 축소로 학습 속도 향상</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -10194,7 +10194,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>SD-v2.1-base를 지식증류로 압축, 배치 축소로 학습 속도를 높인 경량 텍스트-이미지 모델</t>
+          <t>SD-v2.1-base를 지식증류로 압축한 Tiny 크기 경량 텍스트-이미지 모델, 배치 축소로 학습 속도 향상</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -11169,7 +11169,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>SD v1.4 대비 0.1% 미만 데이터만으로 지식증류해 유사 품질을 내는 경량 텍스트-이미지 모델</t>
+          <t>SD v1.4 대비 0.1% 미만 데이터만으로 지식증류한 Base 크기 경량 텍스트-이미지 모델</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -11254,7 +11254,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>이전 대비 10배 많은 LAION 데이터로 사전학습해 이미지 생성 품질 향상, 경량 텍스트-이미지 모델</t>
+          <t>이전 대비 10배 많은 LAION 데이터로 사전학습한 Base 크기 경량 텍스트-이미지 모델, 이미지 생성 품질 향상</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -11339,7 +11339,7 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>SD v1.4 대비 0.1% 미만 데이터만으로 지식증류해 유사 품질을 내는 경량 텍스트-이미지 모델</t>
+          <t>SD v1.4 대비 0.1% 미만 데이터만으로 지식증류한 Small 크기 경량 텍스트-이미지 모델</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
@@ -11424,7 +11424,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>이전 대비 10배 많은 LAION 데이터로 사전학습해 이미지 생성 품질 향상, 경량 텍스트-이미지 모델</t>
+          <t>이전 대비 10배 많은 LAION 데이터로 사전학습한 Small 크기 경량 텍스트-이미지 모델, 이미지 생성 품질 향상</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -11594,7 +11594,7 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>이전 대비 10배 많은 LAION 데이터로 사전학습해 이미지 생성 품질 향상, 경량 텍스트-이미지 모델</t>
+          <t>이전 대비 10배 많은 LAION 데이터로 사전학습한 Tiny 크기 경량 텍스트-이미지 모델, 이미지 생성 품질 향상</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
@@ -12720,7 +12720,7 @@
       <c r="E136" t="inlineStr"/>
       <c r="F136" t="inlineStr">
         <is>
-          <t>한국어 RAG(검색증강생성) 전용 데이터셋으로 QLoRA 파인튜닝되어 RAG 기반 한국어 질의응답에 적합</t>
+          <t>한국어 RAG 전용 데이터셋으로 QLoRA 파인튜닝한 v2.1, RAG 기반 한국어 질의응답에 적합</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
@@ -12805,7 +12805,7 @@
       <c r="E137" t="inlineStr"/>
       <c r="F137" t="inlineStr">
         <is>
-          <t>한국어 RAG(검색증강생성) 전용 데이터셋으로 QLoRA 파인튜닝되어 RAG 기반 한국어 질의응답에 적합</t>
+          <t>한국어 RAG 전용 데이터셋으로 QLoRA 파인튜닝한 v2.0, RAG 기반 한국어 질의응답에 적합</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
@@ -12890,7 +12890,7 @@
       <c r="E138" t="inlineStr"/>
       <c r="F138" t="inlineStr">
         <is>
-          <t>한국어 RAG(검색증강생성) 전용 데이터셋으로 QLoRA 파인튜닝되어 RAG 기반 한국어 질의응답에 적합</t>
+          <t>한국어 RAG 전용 데이터셋으로 QLoRA 파인튜닝한 v1.1, RAG 기반 한국어 질의응답에 적합</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
@@ -12975,7 +12975,7 @@
       <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr">
         <is>
-          <t>한국어 RAG(검색증강생성) 전용 데이터셋으로 QLoRA 파인튜닝되어 RAG 기반 한국어 질의응답에 적합</t>
+          <t>한국어 RAG 전용 데이터셋으로 QLoRA 파인튜닝한 v1.15, RAG 기반 한국어 질의응답에 적합</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
@@ -16691,7 +16691,7 @@
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>한국어 어휘를 확장 학습해 한국어 능력을 강화한 베이스 모델로, 추가 파인튜닝의 기반으로 적합합니다.</t>
+          <t>EEVE 방식으로 한국어 어휘를 확장 학습한 베이스 모델, 추가 파인튜닝의 기반으로 적합</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
@@ -17156,7 +17156,7 @@
       <c r="E186" t="inlineStr"/>
       <c r="F186" t="inlineStr">
         <is>
-          <t>한국어 어휘를 확장 학습해 한국어 능력을 강화한 베이스 모델로, 추가 파인튜닝의 기반으로 적합합니다.</t>
+          <t>SOLAR 기반으로 한국어 어휘를 확장 학습한 KoSOLAR 베이스 모델, 추가 파인튜닝의 기반으로 적합</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
@@ -18268,7 +18268,7 @@
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>OCR·그라운딩·레퍼링을 지원하는 한영 VLM으로 문서·이미지 이해 작업에 적합</t>
+          <t>OCR·그라운딩·레퍼링을 지원하는 한영 VLM(원본 구조), 문서·이미지 이해 작업에 적합</t>
         </is>
       </c>
       <c r="G198" t="inlineStr">
@@ -18357,7 +18357,7 @@
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>OCR·그라운딩·레퍼링을 지원하는 한영 VLM으로 문서·이미지 이해 작업에 적합</t>
+          <t>OCR·그라운딩·레퍼링을 지원하는 한영 VLM의 HF transformers 호환판, 문서·이미지 이해 작업에 적합</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
@@ -19938,7 +19938,7 @@
       <c r="E216" t="inlineStr"/>
       <c r="F216" t="inlineStr">
         <is>
-          <t>Kanana-2 미드트레이닝 체크포인트, 32.5B 이전모델보다 적은 활성파라미터로 32K 문맥·수학·코딩 성능 향상</t>
+          <t>Kanana-2 30B-A3B의 미드트레이닝 체크포인트(2601), base 대비 추가 학습분 반영해 성능 향상</t>
         </is>
       </c>
       <c r="G216" t="inlineStr">
@@ -20239,7 +20239,7 @@
       <c r="E219" t="inlineStr"/>
       <c r="F219" t="inlineStr">
         <is>
-          <t>Kanana-2 미드트레이닝 체크포인트, 32.5B 이전모델보다 적은 활성파라미터로 32K 문맥·수학·코딩 성능 향상</t>
+          <t>Kanana-2 30B-A3B 베이스 모델, 32.5B 이전모델보다 적은 활성파라미터로 32K 문맥·수학·코딩 성능 향상</t>
         </is>
       </c>
       <c r="G219" t="inlineStr">
@@ -20910,7 +20910,7 @@
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>이전 버전 대비 코딩·수학·함수호출 능력 대폭 강화, 32K(YaRN 128K) 문맥 지원해 긴 문서 처리에 적합</t>
+          <t>이전 버전 대비 코딩·수학·함수호출 능력 대폭 강화한 2.1B 베이스, 32K(YaRN 128K) 문맥의 긴 문서 처리에 적합</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
@@ -21009,7 +21009,7 @@
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>이전 버전 대비 코딩·수학·함수호출 능력 강화된 인스트럭트 모델, 32K 문맥 지원해 실전 대화·툴콜에 적합</t>
+          <t>이전 버전 대비 코딩·수학·함수호출 능력 강화한 2.1B 인스트럭트, 32K 문맥 지원해 실전 대화·툴콜에 적합</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
@@ -21108,7 +21108,7 @@
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>이전 버전 대비 코딩·수학·함수호출 능력 대폭 강화, 32K(YaRN 128K) 문맥 지원해 긴 문서 처리에 적합</t>
+          <t>이전 버전 대비 코딩·수학·함수호출 능력 대폭 강화한 8B 베이스, 32K(YaRN 128K) 문맥의 긴 문서 처리에 적합</t>
         </is>
       </c>
       <c r="G228" t="inlineStr">
@@ -21207,7 +21207,7 @@
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>이전 버전 대비 코딩·수학·함수호출 능력 강화된 인스트럭트 모델, 32K 문맥 지원해 실전 대화·툴콜에 적합</t>
+          <t>이전 버전 대비 코딩·수학·함수호출 능력 강화한 8B 인스트럭트, 32K 문맥 지원해 실전 대화·툴콜에 적합</t>
         </is>
       </c>
       <c r="G229" t="inlineStr">
@@ -24473,7 +24473,7 @@
       <c r="E265" t="inlineStr"/>
       <c r="F265" t="inlineStr">
         <is>
-          <t>영어 데이터만으로 학습했음에도 한국어 시각추론에서 LLaVA 대비 우수, 다국어 VLM 연구에 적합</t>
+          <t>영어 데이터만으로 학습했음에도 한국어 시각추론에서 LLaVA 대비 우수(BF16), 다국어 VLM 연구에 적합</t>
         </is>
       </c>
       <c r="G265" t="inlineStr">
@@ -24566,7 +24566,7 @@
       <c r="E266" t="inlineStr"/>
       <c r="F266" t="inlineStr">
         <is>
-          <t>영어 데이터만으로 학습했음에도 한국어 시각추론에서 LLaVA 대비 우수, 다국어 VLM 연구에 적합</t>
+          <t>영어 데이터만으로 학습했음에도 한국어 시각추론에서 LLaVA 대비 우수, FP16 변환판, 다국어 VLM 연구에 적합</t>
         </is>
       </c>
       <c r="G266" t="inlineStr">
@@ -26071,7 +26071,7 @@
       <c r="E283" t="inlineStr"/>
       <c r="F283" t="inlineStr">
         <is>
-          <t>MRL 지원으로 임베딩 차원 축소가 가능해 유연한 의미 검색·유사도 매칭에 적합</t>
+          <t>MRL 지원으로 임베딩 차원 축소가 가능한 0.6B 임베딩 모델, 유연한 의미 검색·유사도 매칭에 적합</t>
         </is>
       </c>
       <c r="G283" t="inlineStr">
@@ -26156,7 +26156,7 @@
       <c r="E284" t="inlineStr"/>
       <c r="F284" t="inlineStr">
         <is>
-          <t>MRL 지원으로 임베딩 차원 축소가 가능해 유연한 의미 검색·유사도 매칭에 적합</t>
+          <t>MRL 지원으로 임베딩 차원 축소가 가능한 4B 임베딩 모델, 유연한 의미 검색·유사도 매칭에 적합</t>
         </is>
       </c>
       <c r="G284" t="inlineStr">
@@ -26241,7 +26241,7 @@
       <c r="E285" t="inlineStr"/>
       <c r="F285" t="inlineStr">
         <is>
-          <t>MRL 지원으로 임베딩 차원 축소가 가능해 유연한 의미 검색·유사도 매칭에 적합</t>
+          <t>MRL 지원으로 임베딩 차원 축소가 가능한 8B 임베딩 모델, 유연한 의미 검색·유사도 매칭에 적합</t>
         </is>
       </c>
       <c r="G285" t="inlineStr">
@@ -26326,7 +26326,7 @@
       <c r="E286" t="inlineStr"/>
       <c r="F286" t="inlineStr">
         <is>
-          <t>쿼리-문서 관련도 점수를 산출해 RAG·검색 파이프라인의 재순위화 단계에 적합</t>
+          <t>쿼리-문서 관련도 점수를 산출하는 0.6B 리랭커, RAG·검색 파이프라인의 재순위화 단계에 적합</t>
         </is>
       </c>
       <c r="G286" t="inlineStr">
@@ -26411,7 +26411,7 @@
       <c r="E287" t="inlineStr"/>
       <c r="F287" t="inlineStr">
         <is>
-          <t>쿼리-문서 관련도 점수를 산출해 RAG·검색 파이프라인의 재순위화 단계에 적합</t>
+          <t>쿼리-문서 관련도 점수를 산출하는 4B 리랭커, RAG·검색 파이프라인의 재순위화 단계에 적합</t>
         </is>
       </c>
       <c r="G287" t="inlineStr">
@@ -26496,7 +26496,7 @@
       <c r="E288" t="inlineStr"/>
       <c r="F288" t="inlineStr">
         <is>
-          <t>쿼리-문서 관련도 점수를 산출해 RAG·검색 파이프라인의 재순위화 단계에 적합</t>
+          <t>쿼리-문서 관련도 점수를 산출하는 8B 리랭커, RAG·검색 파이프라인의 재순위화 단계에 적합</t>
         </is>
       </c>
       <c r="G288" t="inlineStr">
@@ -26581,7 +26581,7 @@
       <c r="E289" t="inlineStr"/>
       <c r="F289" t="inlineStr">
         <is>
-          <t>OCR·문서 및 차트 분석·공간추론·영상이해에 강점이 있어 시각 문서 처리 작업에 적합</t>
+          <t>OCR·문서 및 차트 분석·공간추론·영상이해에 강점 있는 2B VLM, 시각 문서 처리 작업에 적합</t>
         </is>
       </c>
       <c r="G289" t="inlineStr">
@@ -26666,7 +26666,7 @@
       <c r="E290" t="inlineStr"/>
       <c r="F290" t="inlineStr">
         <is>
-          <t>OCR·문서 및 차트 분석·공간추론·영상이해에 강점이 있어 시각 문서 처리 작업에 적합</t>
+          <t>OCR·문서 및 차트 분석·공간추론·영상이해에 강점 있는 32B VLM, 시각 문서 처리 작업에 적합</t>
         </is>
       </c>
       <c r="G290" t="inlineStr">
@@ -26751,7 +26751,7 @@
       <c r="E291" t="inlineStr"/>
       <c r="F291" t="inlineStr">
         <is>
-          <t>OCR·문서 및 차트 분석·공간추론·영상이해에 강점이 있어 시각 문서 처리 작업에 적합</t>
+          <t>OCR·문서 및 차트 분석·공간추론·영상이해에 강점 있는 4B VLM, 시각 문서 처리 작업에 적합</t>
         </is>
       </c>
       <c r="G291" t="inlineStr">
@@ -30034,7 +30034,7 @@
       <c r="E326" t="inlineStr"/>
       <c r="F326" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 크게 높이면서 정확도는 유지해 경량 배포에 적합</t>
+          <t>Llama-3 8B-Instruct를 FP8 양자화해 추론 효율을 높이면서 정확도는 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="G326" t="inlineStr">
@@ -30137,7 +30137,7 @@
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 크게 높이면서 정확도는 유지해 경량 배포에 적합</t>
+          <t>Llama-3.1 70B-Instruct를 FP8 양자화해 추론 효율을 높이면서 정확도는 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="G327" t="inlineStr">
@@ -30240,7 +30240,7 @@
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 크게 높이면서 정확도는 유지해 경량 배포에 적합</t>
+          <t>Llama-3.1 8B-Instruct를 FP8 양자화해 추론 효율을 높이면서 정확도는 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="G328" t="inlineStr">
@@ -30343,7 +30343,7 @@
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>INT8 양자화로 추론 효율을 크게 높이면서 정확도는 유지해 경량 배포에 적합</t>
+          <t>Llama-3.1 70B-Instruct를 INT8 양자화해 추론 효율을 높이면서 정확도는 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="G329" t="inlineStr">
@@ -30446,7 +30446,7 @@
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>INT8 양자화로 추론 효율을 크게 높이면서 정확도는 유지해 경량 배포에 적합</t>
+          <t>Llama-3.1 8B-Instruct를 INT8 양자화해 추론 효율을 높이면서 정확도는 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="G330" t="inlineStr">
@@ -30545,7 +30545,7 @@
       <c r="E331" t="inlineStr"/>
       <c r="F331" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 크게 높이면서 정확도는 유지해 경량 배포에 적합</t>
+          <t>Llama-3 70B(Base)를 FP8 양자화해 추론 효율을 높이면서 정확도는 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="G331" t="inlineStr">
@@ -30640,7 +30640,7 @@
       <c r="E332" t="inlineStr"/>
       <c r="F332" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 크게 높이면서 정확도는 유지해 경량 배포에 적합</t>
+          <t>Llama-3 8B(Base)를 FP8 양자화해 추론 효율을 높이면서 정확도는 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="G332" t="inlineStr">
@@ -30735,7 +30735,7 @@
       <c r="E333" t="inlineStr"/>
       <c r="F333" t="inlineStr">
         <is>
-          <t>INT8 양자화로 추론 효율을 크게 높이면서 정확도는 유지해 경량 배포에 적합</t>
+          <t>Llama-3 8B(Base)를 INT8 양자화해 추론 효율을 높이면서 정확도는 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="G333" t="inlineStr">
@@ -30830,7 +30830,7 @@
       <c r="E334" t="inlineStr"/>
       <c r="F334" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 크게 높이면서 정확도는 유지해 경량 배포에 적합</t>
+          <t>Llama-3 70B-Instruct를 FP8 양자화해 추론 효율을 높이면서 정확도는 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="G334" t="inlineStr">
@@ -30929,7 +30929,7 @@
       <c r="E335" t="inlineStr"/>
       <c r="F335" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 높이면서 정확도를 유지해 대규모 모델의 경량 배포에 적합하다.</t>
+          <t>Mixtral 8x22B(Base)를 FP8 양자화해 정확도를 유지하며 초대형 모델의 경량 배포에 적합</t>
         </is>
       </c>
       <c r="G335" t="inlineStr">
@@ -31014,7 +31014,7 @@
       <c r="E336" t="inlineStr"/>
       <c r="F336" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 높이면서 정확도를 유지해 대규모 모델의 경량 배포에 적합하다.</t>
+          <t>Mixtral 8x22B-Instruct를 FP8 양자화해 정확도를 유지하며 초대형 모델의 경량 배포에 적합</t>
         </is>
       </c>
       <c r="G336" t="inlineStr">
@@ -31099,7 +31099,7 @@
       <c r="E337" t="inlineStr"/>
       <c r="F337" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 높이면서 정확도를 유지해 경량 배포에 적합하다.</t>
+          <t>Mixtral 8x7B(Base)를 FP8 양자화해 추론 효율을 높이면서 정확도를 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="G337" t="inlineStr">
@@ -31188,7 +31188,7 @@
       </c>
       <c r="F338" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 크게 높이면서 정확도는 유지해 경량 배포에 적합</t>
+          <t>Llama-2 13B-Chat을 FP8 양자화해 추론 효율을 높이면서 정확도는 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="G338" t="inlineStr">
@@ -31287,7 +31287,7 @@
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 크게 높이면서 정확도는 유지해 경량 배포에 적합</t>
+          <t>Llama-2 70B-Chat을 FP8 양자화해 추론 효율을 높이면서 정확도는 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="G339" t="inlineStr">
@@ -31386,7 +31386,7 @@
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 크게 높이면서 정확도는 유지해 경량 배포에 적합</t>
+          <t>Llama-2 7B-Chat을 FP8 양자화해 추론 효율을 높이면서 정확도는 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="G340" t="inlineStr">
@@ -31584,7 +31584,7 @@
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 높이면서 정확도를 유지해 경량 배포에 적합하다.</t>
+          <t>Mistral 7B-Instruct(v0.2)를 FP8 양자화해 추론 효율을 높이면서 정확도를 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="G342" t="inlineStr">
@@ -31671,7 +31671,7 @@
       <c r="E343" t="inlineStr"/>
       <c r="F343" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 높이면서 정확도를 유지해 경량 배포에 적합하다.</t>
+          <t>Mixtral 8x7B-Instruct를 FP8 양자화해 추론 효율을 높이면서 정확도를 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="G343" t="inlineStr">
@@ -32908,7 +32908,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 크게 높이면서 정확도는 유지해 경량 배포에 적합</t>
+          <t>Llama-2 13B-Chat을 FP8 양자화해 추론 효율을 높이면서 정확도는 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -33012,7 +33012,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 크게 높이면서 정확도는 유지해 경량 배포에 적합</t>
+          <t>Llama-2 70B-Chat을 FP8 양자화해 추론 효율을 높이면서 정확도는 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -33116,7 +33116,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 크게 높이면서 정확도는 유지해 경량 배포에 적합</t>
+          <t>Llama-2 7B-Chat을 FP8 양자화해 추론 효율을 높이면서 정확도는 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -33424,7 +33424,7 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 크게 높이면서 정확도는 유지해 경량 배포에 적합</t>
+          <t>Llama-3 70B-Instruct를 FP8 양자화해 추론 효율을 높이면서 정확도는 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -33528,7 +33528,7 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 크게 높이면서 정확도는 유지해 경량 배포에 적합</t>
+          <t>Llama-3 70B(Base)를 FP8 양자화해 추론 효율을 높이면서 정확도는 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -33628,7 +33628,7 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 크게 높이면서 정확도는 유지해 경량 배포에 적합</t>
+          <t>Llama-3 8B-Instruct를 FP8 양자화해 추론 효율을 높이면서 정확도는 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -33732,7 +33732,7 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 크게 높이면서 정확도는 유지해 경량 배포에 적합</t>
+          <t>Llama-3 8B(Base)를 FP8 양자화해 추론 효율을 높이면서 정확도는 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -33832,7 +33832,7 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>INT8 양자화로 추론 효율을 크게 높이면서 정확도는 유지해 경량 배포에 적합</t>
+          <t>Llama-3 8B(Base)를 INT8 양자화해 추론 효율을 높이면서 정확도는 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -33936,7 +33936,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 크게 높이면서 정확도는 유지해 경량 배포에 적합</t>
+          <t>Llama-3.1 70B-Instruct를 FP8 양자화해 추론 효율을 높이면서 정확도는 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -34044,7 +34044,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>INT8 양자화로 추론 효율을 크게 높이면서 정확도는 유지해 경량 배포에 적합</t>
+          <t>Llama-3.1 70B-Instruct를 INT8 양자화해 추론 효율을 높이면서 정확도는 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -34152,7 +34152,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 크게 높이면서 정확도는 유지해 경량 배포에 적합</t>
+          <t>Llama-3.1 8B-Instruct를 FP8 양자화해 추론 효율을 높이면서 정확도는 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -34260,7 +34260,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>INT8 양자화로 추론 효율을 크게 높이면서 정확도는 유지해 경량 배포에 적합</t>
+          <t>Llama-3.1 8B-Instruct를 INT8 양자화해 추론 효율을 높이면서 정확도는 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -34770,7 +34770,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 높이면서 정확도를 유지해 경량 배포에 적합하다.</t>
+          <t>Mistral 7B-Instruct(v0.2)를 FP8 양자화해 추론 효율을 높이면서 정확도를 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -34954,7 +34954,7 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 높이면서 정확도를 유지해 대규모 모델의 경량 배포에 적합하다.</t>
+          <t>Mixtral 8x22B-Instruct를 FP8 양자화해 정확도를 유지하며 초대형 모델의 경량 배포에 적합</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -35044,7 +35044,7 @@
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 높이면서 정확도를 유지해 대규모 모델의 경량 배포에 적합하다.</t>
+          <t>Mixtral 8x22B(Base)를 FP8 양자화해 정확도를 유지하며 초대형 모델의 경량 배포에 적합</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -35134,7 +35134,7 @@
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 높이면서 정확도를 유지해 경량 배포에 적합하다.</t>
+          <t>Mixtral 8x7B-Instruct를 FP8 양자화해 추론 효율을 높이면서 정확도를 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -35224,7 +35224,7 @@
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>FP8 양자화로 추론 효율을 높이면서 정확도를 유지해 경량 배포에 적합하다.</t>
+          <t>Mixtral 8x7B(Base)를 FP8 양자화해 추론 효율을 높이면서 정확도를 유지, 경량 배포에 적합</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -38736,7 +38736,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>고성능 32B 모델을 AWQ 4비트로 양자화해 메모리 절약하며 배포 가능</t>
+          <t>EXAONE-3.5 32B 인스트럭트를 AWQ 4비트로 양자화해 메모리 절약하며 배포 가능</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -39808,7 +39808,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>고성능 32B 모델을 AWQ 4비트로 양자화해 메모리 절약하며 배포 가능</t>
+          <t>EXAONE-4.0 32B를 AWQ 4비트로 양자화해 메모리 절약하며 배포 가능</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -40412,7 +40412,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>문서 이해·한국어 맥락 추론에서 동급 최고 성능인 비전언어모델, 한국어 문서 분석에 적합</t>
+          <t>AWQ 4비트로 양자화한 EXAONE-4.5 VLM, 문서 이해·한국어 맥락 추론에서 동급 최고 성능, 한국어 문서 분석에 적합</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -40520,7 +40520,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>문서 이해·한국어 맥락 추론에서 동급 최고 성능인 비전언어모델, 한국어 문서 분석에 적합</t>
+          <t>FP8로 양자화한 EXAONE-4.5 VLM, 문서 이해·한국어 맥락 추론에서 동급 최고 성능, 한국어 문서 분석에 적합</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -40628,7 +40628,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>문서 이해·한국어 맥락 추론에서 동급 최고 성능인 비전언어모델, 한국어 문서 분석에 적합</t>
+          <t>GGUF로 양자화한 EXAONE-4.5 VLM, 문서 이해·한국어 맥락 추론에서 동급 최고 성능, 한국어 문서 분석에 적합</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -41672,7 +41672,7 @@
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>한국어 RAG(검색증강생성) 전용 데이터셋으로 QLoRA 파인튜닝되어 RAG 기반 한국어 질의응답에 적합</t>
+          <t>한국어 RAG 전용 데이터셋으로 QLoRA 파인튜닝한 v1.1, RAG 기반 한국어 질의응답에 적합</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -41762,7 +41762,7 @@
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
-          <t>한국어 RAG(검색증강생성) 전용 데이터셋으로 QLoRA 파인튜닝되어 RAG 기반 한국어 질의응답에 적합</t>
+          <t>한국어 RAG 전용 데이터셋으로 QLoRA 파인튜닝한 v1.15, RAG 기반 한국어 질의응답에 적합</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -41852,7 +41852,7 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>한국어 RAG(검색증강생성) 전용 데이터셋으로 QLoRA 파인튜닝되어 RAG 기반 한국어 질의응답에 적합</t>
+          <t>한국어 RAG 전용 데이터셋으로 QLoRA 파인튜닝한 v2.0, RAG 기반 한국어 질의응답에 적합</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -41942,7 +41942,7 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>한국어 RAG(검색증강생성) 전용 데이터셋으로 QLoRA 파인튜닝되어 RAG 기반 한국어 질의응답에 적합</t>
+          <t>한국어 RAG 전용 데이터셋으로 QLoRA 파인튜닝한 v2.1, RAG 기반 한국어 질의응답에 적합</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -43512,7 +43512,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>OCR·그라운딩·레퍼링을 지원하는 한영 VLM으로 문서·이미지 이해 작업에 적합</t>
+          <t>OCR·그라운딩·레퍼링을 지원하는 한영 VLM(원본 구조), 문서·이미지 이해 작업에 적합</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
@@ -43606,7 +43606,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>OCR·그라운딩·레퍼링을 지원하는 한영 VLM으로 문서·이미지 이해 작업에 적합</t>
+          <t>OCR·그라운딩·레퍼링을 지원하는 한영 VLM의 HF transformers 호환판, 문서·이미지 이해 작업에 적합</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
@@ -45398,7 +45398,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>GRPO로 다중홉 공간추론에 특화 학습되어 순차적 위치·방향 추론 질의응답에 적합</t>
+          <t>GRPO로 다중홉 공간추론에 특화 학습한 32B 모델, 순차적 위치·방향 추론 질의응답에 적합</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
@@ -45492,7 +45492,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>GRPO로 다중홉 공간추론에 특화 학습되어 순차적 위치·방향 추론 질의응답에 적합</t>
+          <t>GRPO로 다중홉 공간추론에 특화 학습한 4B 모델, 순차적 위치·방향 추론 질의응답에 적합</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
@@ -45586,7 +45586,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>GRPO로 다중홉 공간추론에 특화 학습되어 순차적 위치·방향 추론 질의응답에 적합</t>
+          <t>GRPO로 다중홉 공간추론에 특화 학습한 8B 모델, 순차적 위치·방향 추론 질의응답에 적합</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
@@ -45680,7 +45680,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>Gemma 기반 VLM에 이미지 안전분류(20종) 기능을 내장, 유해 콘텐츠 탐지·모더레이션에 적합</t>
+          <t>Gemma 12B 기반 VLM에 이미지 안전분류(20종) 기능을 내장, 유해 콘텐츠 탐지·모더레이션에 적합</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
@@ -45774,7 +45774,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>Gemma 기반 VLM에 이미지 안전분류(20종) 기능을 내장, 유해 콘텐츠 탐지·모더레이션에 적합</t>
+          <t>Gemma 27B 기반 VLM에 이미지 안전분류(20종) 기능을 내장, 유해 콘텐츠 탐지·모더레이션에 적합</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
@@ -45868,7 +45868,7 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>Qwen2.5-VL 기반에 이미지 안전분류(20종) 기능을 내장, 유해 콘텐츠 탐지·모더레이션에 적합</t>
+          <t>Qwen2.5-VL 32B 기반에 이미지 안전분류(20종) 기능을 내장, 유해 콘텐츠 탐지·모더레이션에 적합</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
@@ -45962,7 +45962,7 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>Qwen2.5-VL 기반에 이미지 안전분류(20종) 기능을 내장, 유해 콘텐츠 탐지·모더레이션에 적합</t>
+          <t>Qwen2.5-VL 7B 기반에 이미지 안전분류(20종) 기능을 내장, 유해 콘텐츠 탐지·모더레이션에 적합</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
@@ -47214,7 +47214,7 @@
       <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr">
         <is>
-          <t>MRL 지원으로 임베딩 차원 축소가 가능해 유연한 의미 검색·유사도 매칭에 적합</t>
+          <t>MRL 지원으로 임베딩 차원 축소가 가능한 0.6B 임베딩 모델, 유연한 의미 검색·유사도 매칭에 적합</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
@@ -47304,7 +47304,7 @@
       <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr">
         <is>
-          <t>MRL 지원으로 임베딩 차원 축소가 가능해 유연한 의미 검색·유사도 매칭에 적합</t>
+          <t>MRL 지원으로 임베딩 차원 축소가 가능한 4B 임베딩 모델, 유연한 의미 검색·유사도 매칭에 적합</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
@@ -47394,7 +47394,7 @@
       <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr">
         <is>
-          <t>MRL 지원으로 임베딩 차원 축소가 가능해 유연한 의미 검색·유사도 매칭에 적합</t>
+          <t>MRL 지원으로 임베딩 차원 축소가 가능한 8B 임베딩 모델, 유연한 의미 검색·유사도 매칭에 적합</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
@@ -47484,7 +47484,7 @@
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
         <is>
-          <t>쿼리-문서 관련도 점수를 산출해 RAG·검색 파이프라인의 재순위화 단계에 적합</t>
+          <t>쿼리-문서 관련도 점수를 산출하는 0.6B 리랭커, RAG·검색 파이프라인의 재순위화 단계에 적합</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
@@ -47574,7 +47574,7 @@
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr">
         <is>
-          <t>쿼리-문서 관련도 점수를 산출해 RAG·검색 파이프라인의 재순위화 단계에 적합</t>
+          <t>쿼리-문서 관련도 점수를 산출하는 4B 리랭커, RAG·검색 파이프라인의 재순위화 단계에 적합</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
@@ -47664,7 +47664,7 @@
       <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr">
         <is>
-          <t>쿼리-문서 관련도 점수를 산출해 RAG·검색 파이프라인의 재순위화 단계에 적합</t>
+          <t>쿼리-문서 관련도 점수를 산출하는 8B 리랭커, RAG·검색 파이프라인의 재순위화 단계에 적합</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
@@ -47754,7 +47754,7 @@
       <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr">
         <is>
-          <t>OCR·문서 및 차트 분석·공간추론·영상이해에 강점이 있어 시각 문서 처리 작업에 적합</t>
+          <t>OCR·문서 및 차트 분석·공간추론·영상이해에 강점 있는 2B VLM, 시각 문서 처리 작업에 적합</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
@@ -47844,7 +47844,7 @@
       <c r="F165" t="inlineStr"/>
       <c r="G165" t="inlineStr">
         <is>
-          <t>OCR·문서 및 차트 분석·공간추론·영상이해에 강점이 있어 시각 문서 처리 작업에 적합</t>
+          <t>OCR·문서 및 차트 분석·공간추론·영상이해에 강점 있는 32B VLM, 시각 문서 처리 작업에 적합</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
@@ -47934,7 +47934,7 @@
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
-          <t>OCR·문서 및 차트 분석·공간추론·영상이해에 강점이 있어 시각 문서 처리 작업에 적합</t>
+          <t>OCR·문서 및 차트 분석·공간추론·영상이해에 강점 있는 4B VLM, 시각 문서 처리 작업에 적합</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
@@ -48298,7 +48298,7 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>CoT Collection 184만 rationale 학습, Flan-T5보다 CoT 추론 우수해 제로샷 과제 해결에 적합</t>
+          <t>CoT Collection 184만 rationale로 학습한 11B 모델, Flan-T5보다 CoT 추론 우수해 제로샷 과제에 적합</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
@@ -48388,7 +48388,7 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>CoT Collection 184만 rationale 학습, Flan-T5보다 CoT 추론 우수해 제로샷 과제 해결에 적합</t>
+          <t>CoT Collection 184만 rationale로 학습한 3B 모델, Flan-T5보다 CoT 추론 우수해 제로샷 과제에 적합</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
@@ -48478,7 +48478,7 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>mT5 인코더와 Code Llama를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
+          <t>mT5 인코더와 Code Llama(약 15B)를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
@@ -48568,7 +48568,7 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>mT5 인코더와 Code Llama를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
+          <t>mT5 인코더와 Code Llama(약 20B)를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
@@ -48658,7 +48658,7 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>mT5 인코더와 Code Llama를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
+          <t>mT5 인코더와 Code Llama(약 9B)를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
@@ -49216,7 +49216,7 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>mT5 인코더와 대상 LM을 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
+          <t>mT5 인코더와 Llama2(약 9B)를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
@@ -49306,7 +49306,7 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>mT5 인코더와 대상 LM을 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
+          <t>mT5 인코더와 Llemma(약 9B)를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
@@ -49396,7 +49396,7 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>mT5 인코더와 대상 LM을 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
+          <t>mT5 인코더와 MetaMath(약 15B)를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
@@ -49486,7 +49486,7 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>mT5 인코더와 대상 LM을 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
+          <t>mT5 인코더와 MetaMath(약 20B)를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
@@ -49576,7 +49576,7 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>mT5 인코더와 대상 LM을 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
+          <t>mT5 인코더와 MetaMath(약 9B)를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
@@ -49960,7 +49960,7 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>mT5 인코더와 대상 LM을 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
+          <t>mT5 인코더와 Orca2(약 15B)를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
@@ -50050,7 +50050,7 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>mT5 인코더와 대상 LM을 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
+          <t>mT5 인코더와 Orca2(약 20B)를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
@@ -50140,7 +50140,7 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>mT5 인코더와 대상 LM을 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
+          <t>mT5 인코더와 Orca2(약 9B)를 결합, 다국어 데이터 없이도 다국어 추론 과제 해결에 강점</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
@@ -51040,7 +51040,7 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>이전 버전 대비 코딩·수학·함수호출 능력 대폭 강화, 32K(YaRN 128K) 문맥 지원해 긴 문서 처리에 적합</t>
+          <t>이전 버전 대비 코딩·수학·함수호출 능력 대폭 강화한 2.1B 베이스, 32K(YaRN 128K) 문맥의 긴 문서 처리에 적합</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
@@ -51144,7 +51144,7 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>이전 버전 대비 코딩·수학·함수호출 능력 강화된 인스트럭트 모델, 32K 문맥 지원해 실전 대화·툴콜에 적합</t>
+          <t>이전 버전 대비 코딩·수학·함수호출 능력 강화한 2.1B 인스트럭트, 32K 문맥 지원해 실전 대화·툴콜에 적합</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
@@ -51248,7 +51248,7 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>이전 버전 대비 코딩·수학·함수호출 능력 대폭 강화, 32K(YaRN 128K) 문맥 지원해 긴 문서 처리에 적합</t>
+          <t>이전 버전 대비 코딩·수학·함수호출 능력 대폭 강화한 8B 베이스, 32K(YaRN 128K) 문맥의 긴 문서 처리에 적합</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
@@ -51352,7 +51352,7 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>이전 버전 대비 코딩·수학·함수호출 능력 강화된 인스트럭트 모델, 32K 문맥 지원해 실전 대화·툴콜에 적합</t>
+          <t>이전 버전 대비 코딩·수학·함수호출 능력 강화한 8B 인스트럭트, 32K 문맥 지원해 실전 대화·툴콜에 적합</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
@@ -51556,7 +51556,7 @@
       <c r="F205" t="inlineStr"/>
       <c r="G205" t="inlineStr">
         <is>
-          <t>Kanana-2 미드트레이닝 체크포인트, 32.5B 이전모델보다 적은 활성파라미터로 32K 문맥·수학·코딩 성능 향상</t>
+          <t>Kanana-2 30B-A3B 베이스 모델, 32.5B 이전모델보다 적은 활성파라미터로 32K 문맥·수학·코딩 성능 향상</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
@@ -51976,7 +51976,7 @@
       <c r="F209" t="inlineStr"/>
       <c r="G209" t="inlineStr">
         <is>
-          <t>Kanana-2 미드트레이닝 체크포인트, 32.5B 이전모델보다 적은 활성파라미터로 32K 문맥·수학·코딩 성능 향상</t>
+          <t>Kanana-2 30B-A3B의 미드트레이닝 체크포인트(2601), base 대비 추가 학습분 반영해 성능 향상</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
@@ -53276,7 +53276,7 @@
       </c>
       <c r="G222" t="inlineStr">
         <is>
-          <t>대화체 음성을 실시간에 가깝게 생성하고 웃음·기침 등 비언어적 표현까지 지원, 리서치·교육용 대화형 TTS에 적합</t>
+          <t>대화체 음성을 실시간에 가깝게 생성, 웃음·기침 등 비언어적 표현까지 지원하는 리서치·교육용 대화형 TTS 초기판</t>
         </is>
       </c>
       <c r="H222" t="inlineStr">
@@ -53362,7 +53362,7 @@
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t>대화체 음성을 실시간에 가깝게 생성하고 웃음·기침 등 비언어적 표현까지 지원, 리서치·교육용 대화형 TTS에 적합</t>
+          <t>대화체 음성을 실시간에 가깝게 생성, 웃음·기침 등 비언어적 표현까지 지원하는 리서치·교육용 대화형 TTS 0626 개정판</t>
         </is>
       </c>
       <c r="H223" t="inlineStr">
@@ -53448,7 +53448,7 @@
       <c r="F224" t="inlineStr"/>
       <c r="G224" t="inlineStr">
         <is>
-          <t>문장 전체 없이 실시간 스트리밍으로 대화 음성을 생성해 실시간 음성 대화 시스템에 적합</t>
+          <t>문장 전체 없이 실시간 스트리밍으로 대화 음성을 생성하는 1B 모델, 실시간 음성 대화 시스템에 적합</t>
         </is>
       </c>
       <c r="H224" t="inlineStr">
@@ -53530,7 +53530,7 @@
       <c r="F225" t="inlineStr"/>
       <c r="G225" t="inlineStr">
         <is>
-          <t>문장 전체 없이 실시간 스트리밍으로 대화 음성을 생성해 실시간 음성 대화 시스템에 적합</t>
+          <t>문장 전체 없이 실시간 스트리밍으로 대화 음성을 생성하는 2B 모델, 실시간 음성 대화 시스템에 적합</t>
         </is>
       </c>
       <c r="H225" t="inlineStr">
@@ -55096,7 +55096,7 @@
       </c>
       <c r="G241" t="inlineStr">
         <is>
-          <t>SD v1.4 대비 0.1% 미만 데이터만으로 지식증류해 유사 품질을 내는 경량 텍스트-이미지 모델</t>
+          <t>SD v1.4 대비 0.1% 미만 데이터만으로 지식증류한 Base 크기 경량 텍스트-이미지 모델</t>
         </is>
       </c>
       <c r="H241" t="inlineStr">
@@ -55186,7 +55186,7 @@
       </c>
       <c r="G242" t="inlineStr">
         <is>
-          <t>이전 대비 10배 많은 LAION 데이터로 사전학습해 이미지 생성 품질 향상, 경량 텍스트-이미지 모델</t>
+          <t>이전 대비 10배 많은 LAION 데이터로 사전학습한 Base 크기 경량 텍스트-이미지 모델, 이미지 생성 품질 향상</t>
         </is>
       </c>
       <c r="H242" t="inlineStr">
@@ -55276,7 +55276,7 @@
       </c>
       <c r="G243" t="inlineStr">
         <is>
-          <t>SD v1.4 대비 0.1% 미만 데이터만으로 지식증류해 유사 품질을 내는 경량 텍스트-이미지 모델</t>
+          <t>SD v1.4 대비 0.1% 미만 데이터만으로 지식증류한 Small 크기 경량 텍스트-이미지 모델</t>
         </is>
       </c>
       <c r="H243" t="inlineStr">
@@ -55366,7 +55366,7 @@
       </c>
       <c r="G244" t="inlineStr">
         <is>
-          <t>이전 대비 10배 많은 LAION 데이터로 사전학습해 이미지 생성 품질 향상, 경량 텍스트-이미지 모델</t>
+          <t>이전 대비 10배 많은 LAION 데이터로 사전학습한 Small 크기 경량 텍스트-이미지 모델, 이미지 생성 품질 향상</t>
         </is>
       </c>
       <c r="H244" t="inlineStr">
@@ -55546,7 +55546,7 @@
       </c>
       <c r="G246" t="inlineStr">
         <is>
-          <t>이전 대비 10배 많은 LAION 데이터로 사전학습해 이미지 생성 품질 향상, 경량 텍스트-이미지 모델</t>
+          <t>이전 대비 10배 많은 LAION 데이터로 사전학습한 Tiny 크기 경량 텍스트-이미지 모델, 이미지 생성 품질 향상</t>
         </is>
       </c>
       <c r="H246" t="inlineStr">
@@ -55636,7 +55636,7 @@
       </c>
       <c r="G247" t="inlineStr">
         <is>
-          <t>SD-v2.1-base를 지식증류로 압축, 배치 축소로 학습 속도를 높인 경량 텍스트-이미지 모델</t>
+          <t>SD-v2.1-base를 지식증류로 압축한 Base 크기 경량 텍스트-이미지 모델, 배치 축소로 학습 속도 향상</t>
         </is>
       </c>
       <c r="H247" t="inlineStr">
@@ -55726,7 +55726,7 @@
       </c>
       <c r="G248" t="inlineStr">
         <is>
-          <t>SD-v2.1-base를 지식증류로 압축, 배치 축소로 학습 속도를 높인 경량 텍스트-이미지 모델</t>
+          <t>SD-v2.1-base를 지식증류로 압축한 Small 크기 경량 텍스트-이미지 모델, 배치 축소로 학습 속도 향상</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
@@ -55816,7 +55816,7 @@
       </c>
       <c r="G249" t="inlineStr">
         <is>
-          <t>SD-v2.1-base를 지식증류로 압축, 배치 축소로 학습 속도를 높인 경량 텍스트-이미지 모델</t>
+          <t>SD-v2.1-base를 지식증류로 압축한 Tiny 크기 경량 텍스트-이미지 모델, 배치 축소로 학습 속도 향상</t>
         </is>
       </c>
       <c r="H249" t="inlineStr">
@@ -55906,7 +55906,7 @@
       </c>
       <c r="G250" t="inlineStr">
         <is>
-          <t>Vicuna-7B를 프루닝·LoRA로 경량화, GPU 1장으로 수 시간 내 저비용 재학습 가능</t>
+          <t>Vicuna-7B를 프루닝·LoRA로 경량화한 1.5B 버전, GPU 1장으로 수 시간 내 저비용 재학습 가능</t>
         </is>
       </c>
       <c r="H250" t="inlineStr">
@@ -55996,7 +55996,7 @@
       <c r="F251" t="inlineStr"/>
       <c r="G251" t="inlineStr">
         <is>
-          <t>MLC-LLM·WebLLM에서 바로 구동 가능한 포맷으로 변환해 온디바이스·웹 배포에 적합</t>
+          <t>Vicuna 프루닝 모델을 MLC 포맷(FP16)으로 변환한 1.5B 버전, 온디바이스·웹 배포에 적합</t>
         </is>
       </c>
       <c r="H251" t="inlineStr">
@@ -56082,7 +56082,7 @@
       <c r="F252" t="inlineStr"/>
       <c r="G252" t="inlineStr">
         <is>
-          <t>MLC-LLM·WebLLM에서 바로 구동 가능한 포맷으로 변환해 온디바이스·웹 배포에 적합</t>
+          <t>Vicuna 프루닝 모델을 MLC용 INT4(q4f16_0)로 양자화한 1.5B 버전, 온디바이스·웹 배포에 적합</t>
         </is>
       </c>
       <c r="H252" t="inlineStr">
@@ -56168,7 +56168,7 @@
       <c r="F253" t="inlineStr"/>
       <c r="G253" t="inlineStr">
         <is>
-          <t>MLC-LLM·WebLLM에서 바로 구동 가능한 포맷으로 변환해 온디바이스·웹 배포에 적합</t>
+          <t>Vicuna 프루닝 모델을 MLC용 INT4(q4f16_1)로 양자화한 1.5B 버전, 온디바이스·웹 배포에 적합</t>
         </is>
       </c>
       <c r="H253" t="inlineStr">
@@ -56258,7 +56258,7 @@
       </c>
       <c r="G254" t="inlineStr">
         <is>
-          <t>Vicuna-7B를 프루닝·LoRA로 경량화, GPU 1장으로 수 시간 내 저비용 재학습 가능</t>
+          <t>Vicuna-7B를 프루닝·LoRA로 경량화한 2.7B 버전, GPU 1장으로 수 시간 내 저비용 재학습 가능</t>
         </is>
       </c>
       <c r="H254" t="inlineStr">
@@ -56348,7 +56348,7 @@
       <c r="F255" t="inlineStr"/>
       <c r="G255" t="inlineStr">
         <is>
-          <t>MLC-LLM·WebLLM에서 바로 구동 가능한 포맷으로 변환해 온디바이스·웹 배포에 적합</t>
+          <t>Vicuna 프루닝 모델을 MLC 포맷(FP16)으로 변환한 2.7B 버전, 온디바이스·웹 배포에 적합</t>
         </is>
       </c>
       <c r="H255" t="inlineStr">
@@ -56434,7 +56434,7 @@
       <c r="F256" t="inlineStr"/>
       <c r="G256" t="inlineStr">
         <is>
-          <t>MLC-LLM·WebLLM에서 바로 구동 가능한 포맷으로 변환해 온디바이스·웹 배포에 적합</t>
+          <t>Vicuna 프루닝 모델을 MLC용 INT4(q4f16_0)로 양자화한 2.7B 버전, 온디바이스·웹 배포에 적합</t>
         </is>
       </c>
       <c r="H256" t="inlineStr">
@@ -56520,7 +56520,7 @@
       <c r="F257" t="inlineStr"/>
       <c r="G257" t="inlineStr">
         <is>
-          <t>MLC-LLM·WebLLM에서 바로 구동 가능한 포맷으로 변환해 온디바이스·웹 배포에 적합</t>
+          <t>Vicuna 프루닝 모델을 MLC용 INT4(q4f16_1)로 양자화한 2.7B 버전, 온디바이스·웹 배포에 적합</t>
         </is>
       </c>
       <c r="H257" t="inlineStr">
@@ -56610,7 +56610,7 @@
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t>Vicuna-7B를 프루닝·LoRA로 경량화, GPU 1장으로 수 시간 내 저비용 재학습 가능</t>
+          <t>Vicuna-7B를 프루닝·LoRA로 경량화한 3.7B 버전, GPU 1장으로 수 시간 내 저비용 재학습 가능</t>
         </is>
       </c>
       <c r="H258" t="inlineStr">
@@ -56700,7 +56700,7 @@
       <c r="F259" t="inlineStr"/>
       <c r="G259" t="inlineStr">
         <is>
-          <t>MLC-LLM·WebLLM에서 바로 구동 가능한 포맷으로 변환해 온디바이스·웹 배포에 적합</t>
+          <t>Vicuna 프루닝 모델을 MLC 포맷(FP16)으로 변환한 3.7B 버전, 온디바이스·웹 배포에 적합</t>
         </is>
       </c>
       <c r="H259" t="inlineStr">
@@ -56786,7 +56786,7 @@
       <c r="F260" t="inlineStr"/>
       <c r="G260" t="inlineStr">
         <is>
-          <t>MLC-LLM·WebLLM에서 바로 구동 가능한 포맷으로 변환해 온디바이스·웹 배포에 적합</t>
+          <t>Vicuna 프루닝 모델을 MLC용 INT4(q4f16_0)로 양자화한 3.7B 버전, 온디바이스·웹 배포에 적합</t>
         </is>
       </c>
       <c r="H260" t="inlineStr">
@@ -56872,7 +56872,7 @@
       <c r="F261" t="inlineStr"/>
       <c r="G261" t="inlineStr">
         <is>
-          <t>MLC-LLM·WebLLM에서 바로 구동 가능한 포맷으로 변환해 온디바이스·웹 배포에 적합</t>
+          <t>Vicuna 프루닝 모델을 MLC용 INT4(q4f16_1)로 양자화한 3.7B 버전, 온디바이스·웹 배포에 적합</t>
         </is>
       </c>
       <c r="H261" t="inlineStr">
@@ -57052,7 +57052,7 @@
       <c r="F263" t="inlineStr"/>
       <c r="G263" t="inlineStr">
         <is>
-          <t>MLC-LLM·WebLLM에서 바로 구동 가능한 포맷으로 변환해 온디바이스·웹 배포에 적합</t>
+          <t>Vicuna 프루닝 모델을 MLC 포맷(FP16)으로 변환한 5.5B 버전, 온디바이스·웹 배포에 적합</t>
         </is>
       </c>
       <c r="H263" t="inlineStr">
@@ -57138,7 +57138,7 @@
       <c r="F264" t="inlineStr"/>
       <c r="G264" t="inlineStr">
         <is>
-          <t>MLC-LLM·WebLLM에서 바로 구동 가능한 포맷으로 변환해 온디바이스·웹 배포에 적합</t>
+          <t>Vicuna 프루닝 모델을 MLC용 INT4(q4f16_0)로 양자화한 5.5B 버전, 온디바이스·웹 배포에 적합</t>
         </is>
       </c>
       <c r="H264" t="inlineStr">
@@ -57224,7 +57224,7 @@
       <c r="F265" t="inlineStr"/>
       <c r="G265" t="inlineStr">
         <is>
-          <t>MLC-LLM·WebLLM에서 바로 구동 가능한 포맷으로 변환해 온디바이스·웹 배포에 적합</t>
+          <t>Vicuna 프루닝 모델을 MLC용 INT4(q4f16_1)로 양자화한 5.5B 버전, 온디바이스·웹 배포에 적합</t>
         </is>
       </c>
       <c r="H265" t="inlineStr">
@@ -61418,7 +61418,7 @@
       <c r="F308" t="inlineStr"/>
       <c r="G308" t="inlineStr">
         <is>
-          <t>영어 데이터만으로 학습했음에도 한국어 시각추론에서 LLaVA 대비 우수, 다국어 VLM 연구에 적합</t>
+          <t>영어 데이터만으로 학습했음에도 한국어 시각추론에서 LLaVA 대비 우수(BF16), 다국어 VLM 연구에 적합</t>
         </is>
       </c>
       <c r="H308" t="inlineStr">
@@ -61516,7 +61516,7 @@
       <c r="F309" t="inlineStr"/>
       <c r="G309" t="inlineStr">
         <is>
-          <t>영어 데이터만으로 학습했음에도 한국어 시각추론에서 LLaVA 대비 우수, 다국어 VLM 연구에 적합</t>
+          <t>영어 데이터만으로 학습했음에도 한국어 시각추론에서 LLaVA 대비 우수, FP16 변환판, 다국어 VLM 연구에 적합</t>
         </is>
       </c>
       <c r="H309" t="inlineStr">
@@ -62946,7 +62946,7 @@
       <c r="F324" t="inlineStr"/>
       <c r="G324" t="inlineStr">
         <is>
-          <t>한국어 어휘를 확장 학습해 한국어 능력을 강화한 베이스 모델로, 추가 파인튜닝의 기반으로 적합합니다.</t>
+          <t>SOLAR 기반으로 한국어 어휘를 확장 학습한 KoSOLAR 베이스 모델, 추가 파인튜닝의 기반으로 적합</t>
         </is>
       </c>
       <c r="H324" t="inlineStr">
@@ -63040,7 +63040,7 @@
       </c>
       <c r="G325" t="inlineStr">
         <is>
-          <t>한국어 어휘를 확장 학습해 한국어 능력을 강화한 베이스 모델로, 추가 파인튜닝의 기반으로 적합합니다.</t>
+          <t>EEVE 방식으로 한국어 어휘를 확장 학습한 베이스 모델, 추가 파인튜닝의 기반으로 적합</t>
         </is>
       </c>
       <c r="H325" t="inlineStr">

</xml_diff>

<commit_message>
Keep major-language names visible instead of collapsing to a bare count
format_languages() previously collapsed any 3+ language model down to
"다국어(N개 언어)", losing whether Korean/English/Japanese/Chinese were
among them -- making it impossible to filter the excel by those in
practice. Now the four major languages are always listed by name when
the source data actually specifies them, with the total count appended
(e.g. "한국어, 영어, 일본어, 중국어, 다국어(32개 언어)"). Falls back to a
bare count only when the source genuinely gives no language-level
list (e.g. a README that just states "102 languages").

Backfilled 85 of the 89 existing collapsed rows by re-querying HF's
card_data.language for each model (same structured source refine.py
already reads, not a new guess) and reformatting with the new rule.
4 rows had no language codes on re-fetch and were left untouched.
Regenerated the excel.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/huggingface_models_2026-07-20.xlsx
+++ b/output/huggingface_models_2026-07-20.xlsx
@@ -1976,7 +1976,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>다국어(102개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(102개 언어)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>다국어(102개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(102개 언어)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -2146,7 +2146,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>다국어(102개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(102개 언어)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -2231,7 +2231,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>다국어(102개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(102개 언어)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>다국어(102개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(102개 언어)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2401,7 +2401,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>다국어(102개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(102개 언어)</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>다국어(102개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(102개 언어)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2571,7 +2571,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>다국어(102개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(102개 언어)</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -2656,7 +2656,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>다국어(102개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(102개 언어)</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>다국어(102개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(102개 언어)</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -2826,7 +2826,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>다국어(102개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(102개 언어)</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -3168,7 +3168,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>다국어(6개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(6개 언어)</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>다국어(6개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(6개 언어)</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -3382,7 +3382,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>다국어(6개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(6개 언어)</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3485,7 +3485,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>다국어(6개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(6개 언어)</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>다국어(6개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(6개 언어)</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -3687,7 +3687,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>다국어(6개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(6개 언어)</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -4661,7 +4661,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -4867,7 +4867,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -4970,7 +4970,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -5061,7 +5061,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -5152,7 +5152,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -5239,7 +5239,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -5330,7 +5330,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -5421,7 +5421,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -5512,7 +5512,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -5599,7 +5599,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -11694,7 +11694,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>다국어(8개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(8개 언어)</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
@@ -14582,7 +14582,7 @@
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>다국어(196개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(196개 언어)</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
@@ -15116,7 +15116,7 @@
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>다국어(31개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(31개 언어)</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
@@ -15189,7 +15189,7 @@
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>다국어(5개 언어)</t>
+          <t>한국어, 영어, 다국어(5개 언어)</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
@@ -15521,7 +15521,7 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>다국어(32개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(32개 언어)</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
@@ -15614,7 +15614,7 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>다국어(32개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(32개 언어)</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
@@ -15707,7 +15707,7 @@
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>다국어(32개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(32개 언어)</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
@@ -15800,7 +15800,7 @@
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>다국어(32개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(32개 언어)</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
@@ -15889,7 +15889,7 @@
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>다국어(32개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(32개 언어)</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
@@ -15982,7 +15982,7 @@
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>다국어(32개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(32개 언어)</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
@@ -16075,7 +16075,7 @@
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>다국어(32개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(32개 언어)</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
@@ -16168,7 +16168,7 @@
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>다국어(32개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(32개 언어)</t>
         </is>
       </c>
       <c r="J175" t="inlineStr">
@@ -16257,7 +16257,7 @@
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>다국어(32개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(32개 언어)</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
@@ -16346,7 +16346,7 @@
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>다국어(32개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(32개 언어)</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
@@ -16431,7 +16431,7 @@
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>다국어(11개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(11개 언어)</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
@@ -16524,7 +16524,7 @@
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>다국어(11개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(11개 언어)</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
@@ -16613,7 +16613,7 @@
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>다국어(11개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(11개 언어)</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
@@ -23700,7 +23700,7 @@
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="J257" t="inlineStr">
@@ -23799,7 +23799,7 @@
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="J258" t="inlineStr">
@@ -23906,7 +23906,7 @@
       </c>
       <c r="I259" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="J259" t="inlineStr">
@@ -24009,7 +24009,7 @@
       </c>
       <c r="I260" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="J260" t="inlineStr">
@@ -24112,7 +24112,7 @@
       </c>
       <c r="I261" t="inlineStr">
         <is>
-          <t>다국어(4개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(4개 언어)</t>
         </is>
       </c>
       <c r="J261" t="inlineStr">
@@ -24197,7 +24197,7 @@
       </c>
       <c r="I262" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="J262" t="inlineStr">
@@ -24282,7 +24282,7 @@
       </c>
       <c r="I263" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="J263" t="inlineStr">
@@ -24385,7 +24385,7 @@
       </c>
       <c r="I264" t="inlineStr">
         <is>
-          <t>다국어(4개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(4개 언어)</t>
         </is>
       </c>
       <c r="J264" t="inlineStr">
@@ -24674,7 +24674,7 @@
       </c>
       <c r="I267" t="inlineStr">
         <is>
-          <t>다국어(4개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(4개 언어)</t>
         </is>
       </c>
       <c r="J267" t="inlineStr">
@@ -24781,7 +24781,7 @@
       </c>
       <c r="I268" t="inlineStr">
         <is>
-          <t>다국어(4개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(4개 언어)</t>
         </is>
       </c>
       <c r="J268" t="inlineStr">
@@ -25244,7 +25244,7 @@
       </c>
       <c r="I273" t="inlineStr">
         <is>
-          <t>다국어(6개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(6개 언어)</t>
         </is>
       </c>
       <c r="J273" t="inlineStr">
@@ -25329,7 +25329,7 @@
       </c>
       <c r="I274" t="inlineStr">
         <is>
-          <t>다국어(8개 언어)</t>
+          <t>영어, 다국어(8개 언어)</t>
         </is>
       </c>
       <c r="J274" t="inlineStr">
@@ -25410,7 +25410,7 @@
       </c>
       <c r="I275" t="inlineStr">
         <is>
-          <t>다국어(8개 언어)</t>
+          <t>영어, 다국어(8개 언어)</t>
         </is>
       </c>
       <c r="J275" t="inlineStr">
@@ -27373,7 +27373,7 @@
       </c>
       <c r="I298" t="inlineStr">
         <is>
-          <t>다국어(11개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(11개 언어)</t>
         </is>
       </c>
       <c r="J298" t="inlineStr">
@@ -27464,7 +27464,7 @@
       </c>
       <c r="I299" t="inlineStr">
         <is>
-          <t>다국어(6개 언어)</t>
+          <t>영어, 일본어, 다국어(6개 언어)</t>
         </is>
       </c>
       <c r="J299" t="inlineStr">
@@ -27567,7 +27567,7 @@
       </c>
       <c r="I300" t="inlineStr">
         <is>
-          <t>다국어(6개 언어)</t>
+          <t>영어, 일본어, 다국어(6개 언어)</t>
         </is>
       </c>
       <c r="J300" t="inlineStr">
@@ -27755,7 +27755,7 @@
       </c>
       <c r="I302" t="inlineStr">
         <is>
-          <t>다국어(24개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(24개 언어)</t>
         </is>
       </c>
       <c r="J302" t="inlineStr">
@@ -30255,7 +30255,7 @@
       </c>
       <c r="I328" t="inlineStr">
         <is>
-          <t>다국어(8개 언어)</t>
+          <t>영어, 다국어(8개 언어)</t>
         </is>
       </c>
       <c r="J328" t="inlineStr">
@@ -30358,7 +30358,7 @@
       </c>
       <c r="I329" t="inlineStr">
         <is>
-          <t>다국어(8개 언어)</t>
+          <t>영어, 다국어(8개 언어)</t>
         </is>
       </c>
       <c r="J329" t="inlineStr">
@@ -30461,7 +30461,7 @@
       </c>
       <c r="I330" t="inlineStr">
         <is>
-          <t>다국어(8개 언어)</t>
+          <t>영어, 다국어(8개 언어)</t>
         </is>
       </c>
       <c r="J330" t="inlineStr">
@@ -31496,7 +31496,7 @@
       </c>
       <c r="I341" t="inlineStr">
         <is>
-          <t>다국어(10개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(10개 언어)</t>
         </is>
       </c>
       <c r="J341" t="inlineStr">
@@ -34059,7 +34059,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>다국어(8개 언어)</t>
+          <t>영어, 다국어(8개 언어)</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -34167,7 +34167,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>다국어(8개 언어)</t>
+          <t>영어, 다국어(8개 언어)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -34275,7 +34275,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>다국어(8개 언어)</t>
+          <t>영어, 다국어(8개 언어)</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -34877,7 +34877,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>다국어(11개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(11개 언어)</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -35521,7 +35521,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>다국어(6개 언어)</t>
+          <t>영어, 일본어, 다국어(6개 언어)</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -35629,7 +35629,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>다국어(6개 언어)</t>
+          <t>영어, 일본어, 다국어(6개 언어)</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -36057,7 +36057,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>다국어(24개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(24개 언어)</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -36373,7 +36373,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>다국어(10개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(10개 언어)</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -39227,7 +39227,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -39335,7 +39335,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -39431,7 +39431,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -39527,7 +39527,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -39619,7 +39619,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -39715,7 +39715,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -39823,7 +39823,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -39919,7 +39919,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -40015,7 +40015,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -40107,7 +40107,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -40203,7 +40203,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -40311,7 +40311,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>다국어(6개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(6개 언어)</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -40427,7 +40427,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>다국어(6개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(6개 언어)</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -40535,7 +40535,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>다국어(6개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(6개 언어)</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -40643,7 +40643,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>다국어(6개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(6개 언어)</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -41063,7 +41063,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>다국어(6개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(6개 언어)</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -41179,7 +41179,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>다국어(6개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(6개 언어)</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -41291,7 +41291,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>다국어(8개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(8개 언어)</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -44299,7 +44299,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>다국어(5개 언어)</t>
+          <t>한국어, 영어, 다국어(5개 언어)</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -44377,7 +44377,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>다국어(31개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(31개 언어)</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -46157,7 +46157,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>다국어(6개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(6개 언어)</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -46335,7 +46335,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>다국어(8개 언어)</t>
+          <t>영어, 다국어(8개 언어)</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -46421,7 +46421,7 @@
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>다국어(8개 언어)</t>
+          <t>영어, 다국어(8개 언어)</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -48493,7 +48493,7 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>다국어(102개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(102개 언어)</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -48583,7 +48583,7 @@
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>다국어(102개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(102개 언어)</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -48673,7 +48673,7 @@
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>다국어(102개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(102개 언어)</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -49231,7 +49231,7 @@
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>다국어(102개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(102개 언어)</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -49321,7 +49321,7 @@
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>다국어(102개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(102개 언어)</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -49411,7 +49411,7 @@
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>다국어(102개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(102개 언어)</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -49501,7 +49501,7 @@
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>다국어(102개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(102개 언어)</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
@@ -49591,7 +49591,7 @@
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>다국어(102개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(102개 언어)</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -49975,7 +49975,7 @@
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>다국어(102개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(102개 언어)</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -50065,7 +50065,7 @@
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>다국어(102개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(102개 언어)</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -50155,7 +50155,7 @@
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>다국어(102개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(102개 언어)</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -59075,7 +59075,7 @@
       </c>
       <c r="J285" t="inlineStr">
         <is>
-          <t>다국어(196개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(196개 언어)</t>
         </is>
       </c>
       <c r="K285" t="inlineStr">
@@ -60385,7 +60385,7 @@
       </c>
       <c r="J298" t="inlineStr">
         <is>
-          <t>다국어(4개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(4개 언어)</t>
         </is>
       </c>
       <c r="K298" t="inlineStr">
@@ -60475,7 +60475,7 @@
       </c>
       <c r="J299" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="K299" t="inlineStr">
@@ -60587,7 +60587,7 @@
       </c>
       <c r="J300" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="K300" t="inlineStr">
@@ -60691,7 +60691,7 @@
       </c>
       <c r="J301" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="K301" t="inlineStr">
@@ -60795,7 +60795,7 @@
       </c>
       <c r="J302" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="K302" t="inlineStr">
@@ -60885,7 +60885,7 @@
       </c>
       <c r="J303" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="K303" t="inlineStr">
@@ -60993,7 +60993,7 @@
       </c>
       <c r="J304" t="inlineStr">
         <is>
-          <t>다국어(3개 언어)</t>
+          <t>한국어, 영어, 일본어, 다국어(3개 언어)</t>
         </is>
       </c>
       <c r="K304" t="inlineStr">
@@ -61105,7 +61105,7 @@
       </c>
       <c r="J305" t="inlineStr">
         <is>
-          <t>다국어(4개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(4개 언어)</t>
         </is>
       </c>
       <c r="K305" t="inlineStr">
@@ -61213,7 +61213,7 @@
       </c>
       <c r="J306" t="inlineStr">
         <is>
-          <t>다국어(4개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(4개 언어)</t>
         </is>
       </c>
       <c r="K306" t="inlineStr">
@@ -61325,7 +61325,7 @@
       </c>
       <c r="J307" t="inlineStr">
         <is>
-          <t>다국어(4개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(4개 언어)</t>
         </is>
       </c>
       <c r="K307" t="inlineStr">
@@ -63737,7 +63737,7 @@
       </c>
       <c r="J332" t="inlineStr">
         <is>
-          <t>다국어(11개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(11개 언어)</t>
         </is>
       </c>
       <c r="K332" t="inlineStr">
@@ -63835,7 +63835,7 @@
       </c>
       <c r="J333" t="inlineStr">
         <is>
-          <t>다국어(32개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(32개 언어)</t>
         </is>
       </c>
       <c r="K333" t="inlineStr">
@@ -63933,7 +63933,7 @@
       </c>
       <c r="J334" t="inlineStr">
         <is>
-          <t>다국어(32개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(32개 언어)</t>
         </is>
       </c>
       <c r="K334" t="inlineStr">
@@ -64027,7 +64027,7 @@
       </c>
       <c r="J335" t="inlineStr">
         <is>
-          <t>다국어(11개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(11개 언어)</t>
         </is>
       </c>
       <c r="K335" t="inlineStr">
@@ -64125,7 +64125,7 @@
       </c>
       <c r="J336" t="inlineStr">
         <is>
-          <t>다국어(32개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(32개 언어)</t>
         </is>
       </c>
       <c r="K336" t="inlineStr">
@@ -64223,7 +64223,7 @@
       </c>
       <c r="J337" t="inlineStr">
         <is>
-          <t>다국어(32개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(32개 언어)</t>
         </is>
       </c>
       <c r="K337" t="inlineStr">
@@ -64321,7 +64321,7 @@
       </c>
       <c r="J338" t="inlineStr">
         <is>
-          <t>다국어(32개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(32개 언어)</t>
         </is>
       </c>
       <c r="K338" t="inlineStr">
@@ -64411,7 +64411,7 @@
       </c>
       <c r="J339" t="inlineStr">
         <is>
-          <t>다국어(11개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(11개 언어)</t>
         </is>
       </c>
       <c r="K339" t="inlineStr">
@@ -64509,7 +64509,7 @@
       </c>
       <c r="J340" t="inlineStr">
         <is>
-          <t>다국어(32개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(32개 언어)</t>
         </is>
       </c>
       <c r="K340" t="inlineStr">
@@ -64607,7 +64607,7 @@
       </c>
       <c r="J341" t="inlineStr">
         <is>
-          <t>다국어(32개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(32개 언어)</t>
         </is>
       </c>
       <c r="K341" t="inlineStr">
@@ -64701,7 +64701,7 @@
       </c>
       <c r="J342" t="inlineStr">
         <is>
-          <t>다국어(32개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(32개 언어)</t>
         </is>
       </c>
       <c r="K342" t="inlineStr">
@@ -64799,7 +64799,7 @@
       </c>
       <c r="J343" t="inlineStr">
         <is>
-          <t>다국어(32개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(32개 언어)</t>
         </is>
       </c>
       <c r="K343" t="inlineStr">
@@ -64897,7 +64897,7 @@
       </c>
       <c r="J344" t="inlineStr">
         <is>
-          <t>다국어(32개 언어)</t>
+          <t>한국어, 영어, 일본어, 중국어, 다국어(32개 언어)</t>
         </is>
       </c>
       <c r="K344" t="inlineStr">

</xml_diff>